<commit_message>
Closeout/closeout.feature - Changes done as per scenarios Closeout_Field_Values.xlsx - Changes done as per scenarios FocusArea_Field_Values.xlsx - Used standard names for automation records FundingSource_Field_Values.xlsx - Used standard names for automation records closeout.properties - Moved Id's to properties files
</commit_message>
<xml_diff>
--- a/src/main/resources/Closeout_Field_Values.xlsx
+++ b/src/main/resources/Closeout_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FB98CD9-7F13-403C-97BE-0E0C956C1964}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD7F92C9-1146-4677-A05D-1AA0D41D4D9B}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20160" windowHeight="8916" activeTab="1" xr2:uid="{53A78F2A-66A3-4C9D-BADA-DECB8EFCEB55}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{53A78F2A-66A3-4C9D-BADA-DECB8EFCEB55}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="49">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -177,6 +177,9 @@
   </si>
   <si>
     <t>ChecklistQuestionPick6__c</t>
+  </si>
+  <si>
+    <t>fieldReason__c</t>
   </si>
 </sst>
 </file>
@@ -535,14 +538,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D63121E-24A7-4605-825A-0B99C45876A1}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -553,7 +556,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -564,7 +567,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -582,14 +585,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81A642DD-5C22-403F-AC5C-036497C62C6C}">
-  <dimension ref="A1:C31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C32"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.6640625" customWidth="1"/>
-    <col min="3" max="3" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.7109375" customWidth="1"/>
+    <col min="3" max="3" width="25.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -600,7 +603,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -611,7 +614,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -622,7 +625,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -633,7 +636,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -644,7 +647,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -655,7 +658,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -666,7 +669,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -677,7 +680,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -688,7 +691,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -699,7 +702,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -710,7 +713,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -721,7 +724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -732,7 +735,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -743,7 +746,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -754,7 +757,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -765,7 +768,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -776,7 +779,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -787,7 +790,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -798,7 +801,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -809,7 +812,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -820,7 +823,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -831,7 +834,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>9</v>
       </c>
@@ -842,7 +845,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -853,7 +856,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -864,7 +867,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>9</v>
       </c>
@@ -875,7 +878,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>9</v>
       </c>
@@ -886,7 +889,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>9</v>
       </c>
@@ -897,7 +900,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>9</v>
       </c>
@@ -908,7 +911,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -919,7 +922,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>9</v>
       </c>
@@ -930,21 +933,33 @@
         <v>16</v>
       </c>
     </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" t="s">
+        <v>48</v>
+      </c>
+      <c r="C32" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D229D022-2CD7-4F3C-BA00-D4F6DB9FA189}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -955,7 +970,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -974,14 +989,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B11CE9E0-A984-444A-96CC-42B957DC3B9C}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -992,7 +1007,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -1003,7 +1018,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>40</v>
       </c>
@@ -1014,7 +1029,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>40</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 1994: created separate feature file for scheduled payment Request
created separate feature file for scheduled payment Request
</commit_message>
<xml_diff>
--- a/src/main/resources/Closeout_Field_Values.xlsx
+++ b/src/main/resources/Closeout_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD7F92C9-1146-4677-A05D-1AA0D41D4D9B}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7A23FF-CE7E-44B0-8D2D-E7FE117AAF19}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{53A78F2A-66A3-4C9D-BADA-DECB8EFCEB55}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{53A78F2A-66A3-4C9D-BADA-DECB8EFCEB55}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="46">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -159,15 +159,6 @@
   </si>
   <si>
     <t>I Agree</t>
-  </si>
-  <si>
-    <t>AggreementDate__c</t>
-  </si>
-  <si>
-    <t>AggreementBy__c</t>
-  </si>
-  <si>
-    <t>Automation SPI</t>
   </si>
   <si>
     <t>Comments5__c</t>
@@ -663,7 +654,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
@@ -850,7 +841,7 @@
         <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C24" t="s">
         <v>16</v>
@@ -938,7 +929,7 @@
         <v>40</v>
       </c>
       <c r="B32" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C32" t="s">
         <v>16</v>
@@ -975,7 +966,7 @@
         <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -988,7 +979,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B11CE9E0-A984-444A-96CC-42B957DC3B9C}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -1018,28 +1009,6 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" t="s">
-        <v>44</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Merged PR 2369: Merge planningmodulenewscenarios to master
</commit_message>
<xml_diff>
--- a/src/main/resources/Closeout_Field_Values.xlsx
+++ b/src/main/resources/Closeout_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7A23FF-CE7E-44B0-8D2D-E7FE117AAF19}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3952959C-4542-4FB1-B903-3EA4A154598F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{53A78F2A-66A3-4C9D-BADA-DECB8EFCEB55}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{53A78F2A-66A3-4C9D-BADA-DECB8EFCEB55}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -158,9 +158,6 @@
     <t>Overview</t>
   </si>
   <si>
-    <t>I Agree</t>
-  </si>
-  <si>
     <t>Comments5__c</t>
   </si>
   <si>
@@ -171,6 +168,9 @@
   </si>
   <si>
     <t>fieldReason__c</t>
+  </si>
+  <si>
+    <t>Checked</t>
   </si>
 </sst>
 </file>
@@ -529,14 +529,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D63121E-24A7-4605-825A-0B99C45876A1}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -547,7 +547,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -558,7 +558,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -577,13 +577,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81A642DD-5C22-403F-AC5C-036497C62C6C}">
   <dimension ref="A1:C32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.7109375" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -594,7 +594,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -605,7 +605,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -616,7 +616,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -627,7 +627,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -638,7 +638,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -649,18 +649,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -671,7 +671,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -682,7 +682,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -693,7 +693,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -704,7 +704,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -715,7 +715,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -737,7 +737,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -748,7 +748,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -759,7 +759,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -770,7 +770,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -781,7 +781,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -792,7 +792,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -803,7 +803,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -814,7 +814,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -825,7 +825,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>9</v>
       </c>
@@ -836,18 +836,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C24" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -858,7 +858,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>9</v>
       </c>
@@ -869,7 +869,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>9</v>
       </c>
@@ -880,7 +880,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>9</v>
       </c>
@@ -891,7 +891,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>9</v>
       </c>
@@ -902,7 +902,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -913,7 +913,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>9</v>
       </c>
@@ -924,12 +924,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>40</v>
       </c>
       <c r="B32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C32" t="s">
         <v>16</v>
@@ -944,13 +944,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D229D022-2CD7-4F3C-BA00-D4F6DB9FA189}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -961,12 +961,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -980,14 +980,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B11CE9E0-A984-444A-96CC-42B957DC3B9C}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -998,7 +998,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed business suite test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Closeout_Field_Values.xlsx
+++ b/src/main/resources/Closeout_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Product Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A732C3A5-3987-4854-B656-4392C87FBB68}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9808803-9027-437C-B49A-0AD62E804F1F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{53A78F2A-66A3-4C9D-BADA-DECB8EFCEB55}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{53A78F2A-66A3-4C9D-BADA-DECB8EFCEB55}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -649,14 +649,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D63121E-24A7-4605-825A-0B99C45876A1}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -667,7 +667,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -678,7 +678,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -691,18 +691,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7BBCD17-F259-4C54-8AFE-639F1178A6AB}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -713,7 +714,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -724,7 +725,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -744,13 +745,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81A642DD-5C22-403F-AC5C-036497C62C6C}">
   <dimension ref="A1:C32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.7109375" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -761,7 +762,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -772,7 +773,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -783,7 +784,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -794,7 +795,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -805,7 +806,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -816,7 +817,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -827,7 +828,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -838,7 +839,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -849,7 +850,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -860,7 +861,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -871,7 +872,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -882,7 +883,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -893,7 +894,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -904,7 +905,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -915,7 +916,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -926,7 +927,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -937,7 +938,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -948,7 +949,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -959,7 +960,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -970,7 +971,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -981,7 +982,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -992,7 +993,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>9</v>
       </c>
@@ -1003,7 +1004,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -1014,7 +1015,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -1025,7 +1026,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>9</v>
       </c>
@@ -1036,7 +1037,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>9</v>
       </c>
@@ -1047,7 +1048,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>9</v>
       </c>
@@ -1058,7 +1059,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>9</v>
       </c>
@@ -1069,7 +1070,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -1080,7 +1081,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>9</v>
       </c>
@@ -1091,7 +1092,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>40</v>
       </c>
@@ -1111,13 +1112,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5F7DE33-22A9-4DFB-A132-6081F21423BE}">
   <dimension ref="A1:C32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1128,7 +1129,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1139,7 +1140,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1150,7 +1151,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1161,7 +1162,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1172,7 +1173,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1183,7 +1184,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1194,7 +1195,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1205,7 +1206,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1216,7 +1217,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1227,7 +1228,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1238,7 +1239,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1249,7 +1250,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1260,7 +1261,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1271,7 +1272,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -1282,7 +1283,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -1293,7 +1294,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -1304,7 +1305,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -1315,7 +1316,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -1326,7 +1327,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -1337,7 +1338,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -1348,7 +1349,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -1359,7 +1360,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>9</v>
       </c>
@@ -1370,7 +1371,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -1381,7 +1382,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -1392,7 +1393,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>9</v>
       </c>
@@ -1403,7 +1404,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>9</v>
       </c>
@@ -1414,7 +1415,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>9</v>
       </c>
@@ -1425,7 +1426,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>9</v>
       </c>
@@ -1436,7 +1437,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -1447,7 +1448,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>9</v>
       </c>
@@ -1458,7 +1459,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>40</v>
       </c>
@@ -1478,13 +1479,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D229D022-2CD7-4F3C-BA00-D4F6DB9FA189}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1495,7 +1496,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -1514,14 +1515,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B11CE9E0-A984-444A-96CC-42B957DC3B9C}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1532,7 +1533,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>40</v>
       </c>

</xml_diff>